<commit_message>
Expand M2 conformance coverage for issue #276 functions
Improves PROPER, SEARCH, COUNTBLANK, COUNTIF, SUMIF, AVERAGEIF test cases:
- PROPER: add coercion (numbers, TRUE/FALSE), error propagation, hyphenated edge
- SEARCH: add ? wildcard, coercion (number search), start-pos edge, more nested
- COUNTBLANK: add zero/FALSE/TRUE non-blank cases, coercion, COUNTA nested
- COUNTIF: add <> operator, ? wildcard, case-insensitive, covers-all nested
- SUMIF: add <> operator, ? wildcard, case-insensitive, coercion
- AVERAGEIF: add <> operator, ? wildcard, >= edge, coercion, nested compare

Regenerated from updated generator scripts in brain/projects/ganit/test-generators/.
All 6 active conformance tests pass; 24 pending remain ignored.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/crates/core/tests/fixtures/m2/Math.xlsx
+++ b/crates/core/tests/fixtures/m2/Math.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="486">
   <si>
     <t>Description</t>
   </si>
@@ -396,6 +396,39 @@
     <t>=COUNTBLANK({"a","b","c"})</t>
   </si>
   <si>
+    <t>zero is not blank -&gt; 0</t>
+  </si>
+  <si>
+    <t>=COUNTBLANK({0})</t>
+  </si>
+  <si>
+    <t>FALSE is not blank -&gt; 0</t>
+  </si>
+  <si>
+    <t>=COUNTBLANK({FALSE})</t>
+  </si>
+  <si>
+    <t>TRUE is not blank -&gt; 0</t>
+  </si>
+  <si>
+    <t>=COUNTBLANK({TRUE})</t>
+  </si>
+  <si>
+    <t>mixed text and blank -&gt; 1</t>
+  </si>
+  <si>
+    <t>=COUNTBLANK({"hello","","world"})</t>
+  </si>
+  <si>
+    <t>coercion: blank among booleans -&gt; 1</t>
+  </si>
+  <si>
+    <t>=COUNTBLANK({TRUE,FALSE,""})</t>
+  </si>
+  <si>
+    <t>coercion</t>
+  </si>
+  <si>
     <t>=COUNTBLANK()</t>
   </si>
   <si>
@@ -405,6 +438,12 @@
     <t>=COUNTBLANK({"",1,"",2})+COUNT({1,2})</t>
   </si>
   <si>
+    <t>nested: COUNTBLANK+COUNTA -&gt; total</t>
+  </si>
+  <si>
+    <t>=COUNTBLANK({"",1,"",2})+COUNTA({"",1,"",2})</t>
+  </si>
+  <si>
     <t>count &gt; 2 in {1..5} -&gt; 3</t>
   </si>
   <si>
@@ -435,10 +474,16 @@
     <t>=COUNTIF({1,2,3,4,5},"&gt;="&amp;2)</t>
   </si>
   <si>
-    <t>wildcard * matches all non-empty -&gt; 5</t>
-  </si>
-  <si>
-    <t>=COUNTIF({1,2,3,4,5},"*")</t>
+    <t>wildcard * matches all text -&gt; 3</t>
+  </si>
+  <si>
+    <t>=COUNTIF({"a","b","c"},"*")</t>
+  </si>
+  <si>
+    <t>not-equal &lt;&gt; criterion -&gt; 4</t>
+  </si>
+  <si>
+    <t>=COUNTIF({1,2,3,2,1},"&lt;&gt;"&amp;2)</t>
   </si>
   <si>
     <t>no matches -&gt; 0</t>
@@ -453,6 +498,24 @@
     <t>=COUNTIF({TRUE,FALSE,FALSE},FALSE)</t>
   </si>
   <si>
+    <t>? wildcard single char ap? -&gt; 2</t>
+  </si>
+  <si>
+    <t>=COUNTIF({"apt","ape","app","bat"},"ap?")</t>
+  </si>
+  <si>
+    <t>count text case-insensitive A matches a</t>
+  </si>
+  <si>
+    <t>=COUNTIF({"a","b","A","c"},"a")</t>
+  </si>
+  <si>
+    <t>coercion: criterion number matches number string</t>
+  </si>
+  <si>
+    <t>=COUNTIF({1,2,3},2)</t>
+  </si>
+  <si>
     <t>=COUNTIF()</t>
   </si>
   <si>
@@ -462,6 +525,12 @@
     <t>=COUNTIF({1,2,3,4,5},"&gt;"&amp;2)*2</t>
   </si>
   <si>
+    <t>nested: COUNTIF+COUNTIF covers all</t>
+  </si>
+  <si>
+    <t>=COUNTIF({1,2,3,4,5},"&gt;"&amp;2)+COUNTIF({1,2,3,4,5},"&lt;="&amp;2)</t>
+  </si>
+  <si>
     <t>single criterion &gt; 2 -&gt; 3</t>
   </si>
   <si>
@@ -474,7 +543,7 @@
     <t>=COUNTIFS({1,2,3,4,5},"&gt;"&amp;1,{1,2,3,4,5},"&lt;"&amp;5)</t>
   </si>
   <si>
-    <t>no matches double criteria</t>
+    <t>no matches double criteria -&gt; 0</t>
   </si>
   <si>
     <t>=COUNTIFS({1,2,3},"&gt;"&amp;5,{1,2,3},"&lt;"&amp;10)</t>
@@ -486,12 +555,30 @@
     <t>=COUNTIFS({1,2,3,2,1},2)</t>
   </si>
   <si>
-    <t>two criteria both equal</t>
+    <t>not-equal &lt;&gt; criterion in COUNTIFS</t>
+  </si>
+  <si>
+    <t>=COUNTIFS({1,2,3,2,1},"&lt;&gt;"&amp;2)</t>
+  </si>
+  <si>
+    <t>two criteria both equal -&gt; 3</t>
   </si>
   <si>
     <t>=COUNTIFS({1,2,3},"&gt;="&amp;1,{1,2,3},"&lt;="&amp;3)</t>
   </si>
   <si>
+    <t>text criterion in COUNTIFS</t>
+  </si>
+  <si>
+    <t>=COUNTIFS({"a","b","a","c"},"a")</t>
+  </si>
+  <si>
+    <t>wildcard * in COUNTIFS</t>
+  </si>
+  <si>
+    <t>=COUNTIFS({"apple","apricot","banana"},"a*")</t>
+  </si>
+  <si>
     <t>=COUNTIFS()</t>
   </si>
   <si>
@@ -501,10 +588,10 @@
     <t>=COUNTIFS({1,2,3,4,5},"&gt;"&amp;2)+COUNTIFS({1,2,3,4,5},"&lt;"&amp;3)</t>
   </si>
   <si>
-    <t>text criterion in COUNTIFS</t>
-  </si>
-  <si>
-    <t>=COUNTIFS({"a","b","a","c"},"a")</t>
+    <t>nested: COUNTIFS inside IF</t>
+  </si>
+  <si>
+    <t>=IF(COUNTIFS({1,2,3,4,5},"&gt;"&amp;4)=1,"yes","no")</t>
   </si>
   <si>
     <t>3 unique from 6 values</t>
@@ -1233,15 +1320,39 @@
     <t>=SUMIF({1,2,3,4,5},3)</t>
   </si>
   <si>
+    <t>not-equal &lt;&gt; criterion -&gt; sum 1+3=4</t>
+  </si>
+  <si>
+    <t>=SUMIF({1,2,3},"&lt;&gt;"&amp;2)</t>
+  </si>
+  <si>
     <t>=SUMIF({1,2,3},"&gt;"&amp;10)</t>
   </si>
   <si>
-    <t>wildcard criterion *</t>
+    <t>wildcard * matches all text</t>
   </si>
   <si>
     <t>=SUMIF({"a","b","c"},"*",{10,20,30})</t>
   </si>
   <si>
+    <t>? wildcard single char: a? matches ab, ac</t>
+  </si>
+  <si>
+    <t>=SUMIF({"ab","ac","ba"},"a?",{10,20,30})</t>
+  </si>
+  <si>
+    <t>case-insensitive text criterion</t>
+  </si>
+  <si>
+    <t>=SUMIF({"Apple","APPLE","banana"},"apple",{10,20,30})</t>
+  </si>
+  <si>
+    <t>coercion: number criterion as string</t>
+  </si>
+  <si>
+    <t>=SUMIF({1,2,3},"2",{10,20,30})</t>
+  </si>
+  <si>
     <t>=SUMIF()</t>
   </si>
   <si>
@@ -1257,6 +1368,12 @@
     <t>=SUMIF({1,2,3},"&gt;"&amp;1,{-10,-20,-30})</t>
   </si>
   <si>
+    <t>nested: ROUND(SUMIF)</t>
+  </si>
+  <si>
+    <t>=ROUND(SUMIF({1.1,2.2,3.3},"&gt;"&amp;2,{10,20,30}),0)</t>
+  </si>
+  <si>
     <t>single criterion sum &gt; 2 -&gt; 12</t>
   </si>
   <si>
@@ -1275,12 +1392,30 @@
     <t>=SUMIFS({1,2,3},{1,2,3},"&gt;"&amp;10)</t>
   </si>
   <si>
+    <t>not-equal &lt;&gt; criterion in SUMIFS</t>
+  </si>
+  <si>
+    <t>=SUMIFS({10,20,30},{1,2,3},"&lt;&gt;"&amp;2)</t>
+  </si>
+  <si>
     <t>exact match criterion</t>
   </si>
   <si>
     <t>=SUMIFS({10,20,30},{1,2,3},2)</t>
   </si>
   <si>
+    <t>wildcard * in SUMIFS</t>
+  </si>
+  <si>
+    <t>=SUMIFS({10,20,30},{"apple","apricot","banana"},"a*")</t>
+  </si>
+  <si>
+    <t>two criteria both must match</t>
+  </si>
+  <si>
+    <t>=SUMIFS({100,200,300,400},{"a","b","a","b"},"a",{1,2,1,2},1)</t>
+  </si>
+  <si>
     <t>=SUMIFS()</t>
   </si>
   <si>
@@ -1290,10 +1425,10 @@
     <t>=SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;3)+SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&lt;"&amp;3)</t>
   </si>
   <si>
-    <t>two criteria both must match</t>
-  </si>
-  <si>
-    <t>=SUMIFS({100,200,300,400},{"a","b","a","b"},"a",{1,2,1,2},1)</t>
+    <t>nested: ROUND(SUMIFS)</t>
+  </si>
+  <si>
+    <t>=ROUND(SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;1,{1,2,3,4,5},"&lt;"&amp;5),0)</t>
   </si>
   <si>
     <t>SUMSQ(3,4) -&gt; 25</t>
@@ -1385,7 +1520,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1410,6 +1545,12 @@
         <bgColor rgb="FFF0F8FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFDE7"/>
+        <bgColor rgb="FFFFFDE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -1417,7 +1558,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1445,6 +1586,13 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf quotePrefix="1" borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1973,10 +2121,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>175</v>
+        <v>204</v>
       </c>
       <c r="C2" s="4">
         <f>DECIMAL("FF",16)</f>
@@ -1988,10 +2136,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>177</v>
+        <v>206</v>
       </c>
       <c r="C3" s="4">
         <f>DECIMAL("1010",2)</f>
@@ -2003,10 +2151,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>178</v>
+        <v>207</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="C4" s="4">
         <f>DECIMAL("10",8)</f>
@@ -2018,10 +2166,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="C5" s="4">
         <f>DECIMAL("Z",36)</f>
@@ -2033,10 +2181,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="C6" s="4">
         <f>DECIMAL("0",10)</f>
@@ -2048,10 +2196,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>184</v>
+        <v>213</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>185</v>
+        <v>214</v>
       </c>
       <c r="C7" s="4">
         <f>DECIMAL("ff",16)</f>
@@ -2063,10 +2211,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>186</v>
+        <v>215</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
       <c r="C8" s="4">
         <f>DECIMAL("1",2)</f>
@@ -2078,10 +2226,10 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>189</v>
+        <v>218</v>
       </c>
       <c r="C9" s="7" t="str">
         <f>DECIMAL("G",16)</f>
@@ -2096,7 +2244,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>DECIMAL()</f>
@@ -2108,10 +2256,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>192</v>
+        <v>221</v>
       </c>
       <c r="C11" s="10" t="str">
         <f>BASE(DECIMAL("FF",16),16)</f>
@@ -2155,10 +2303,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>194</v>
+        <v>223</v>
       </c>
       <c r="C2" s="4">
         <f>FACTDOUBLE(5)</f>
@@ -2170,10 +2318,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="C3" s="4">
         <f>FACTDOUBLE(6)</f>
@@ -2185,10 +2333,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="C4" s="4">
         <f>FACTDOUBLE(1)</f>
@@ -2200,10 +2348,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="C5" s="4">
         <f>FACTDOUBLE(0)</f>
@@ -2215,10 +2363,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
       <c r="C6" s="4">
         <f>FACTDOUBLE(2)</f>
@@ -2230,10 +2378,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="C7" s="4">
         <f>FACTDOUBLE(4)</f>
@@ -2245,10 +2393,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>206</v>
+        <v>235</v>
       </c>
       <c r="C8" s="4">
         <f>FACTDOUBLE(7)</f>
@@ -2260,10 +2408,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>207</v>
+        <v>236</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="C9" s="4">
         <f>FACTDOUBLE(8)</f>
@@ -2275,10 +2423,10 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>FACTDOUBLE(-1)</f>
@@ -2293,7 +2441,7 @@
         <v>27</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>211</v>
+        <v>240</v>
       </c>
       <c r="C11" s="7" t="str">
         <f>FACTDOUBLE()</f>
@@ -2305,10 +2453,10 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>213</v>
+        <v>242</v>
       </c>
       <c r="C12" s="10">
         <f>FACTDOUBLE(5)/FACTDOUBLE(3)</f>
@@ -2352,10 +2500,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>214</v>
+        <v>243</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>215</v>
+        <v>244</v>
       </c>
       <c r="C2" s="4">
         <f>_xlfn.FLOOR.MATH(5.5)</f>
@@ -2367,10 +2515,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>216</v>
+        <v>245</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>217</v>
+        <v>246</v>
       </c>
       <c r="C3" s="4">
         <f>_xlfn.FLOOR.MATH(6,2)</f>
@@ -2382,10 +2530,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
       <c r="C4" s="4">
         <f>_xlfn.FLOOR.MATH(5,2)</f>
@@ -2400,7 +2548,7 @@
         <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>220</v>
+        <v>249</v>
       </c>
       <c r="C5" s="4">
         <f>_xlfn.FLOOR.MATH(0)</f>
@@ -2412,10 +2560,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>221</v>
+        <v>250</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>222</v>
+        <v>251</v>
       </c>
       <c r="C6" s="4">
         <f>_xlfn.FLOOR.MATH(3.9,0.5)</f>
@@ -2427,10 +2575,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>223</v>
+        <v>252</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="C7" s="4">
         <f>_xlfn.FLOOR.MATH(-5.5,1,0)</f>
@@ -2442,10 +2590,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>226</v>
+        <v>255</v>
       </c>
       <c r="C8" s="4">
         <f>_xlfn.FLOOR.MATH(-5.5,1,1)</f>
@@ -2457,10 +2605,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>227</v>
+        <v>256</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="C9" s="4">
         <f>_xlfn.FLOOR.MATH(-4.1,2,0)</f>
@@ -2475,7 +2623,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>229</v>
+        <v>258</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>_xlfn.FLOOR.MATH()</f>
@@ -2487,10 +2635,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>231</v>
+        <v>260</v>
       </c>
       <c r="C11" s="10">
         <f>_xlfn.FLOOR.MATH(PI())</f>
@@ -2534,10 +2682,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>214</v>
+        <v>243</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="C2" s="4">
         <f>_xlfn.FLOOR.PRECISE(5.5)</f>
@@ -2549,10 +2697,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>233</v>
+        <v>262</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>234</v>
+        <v>263</v>
       </c>
       <c r="C3" s="4">
         <f>_xlfn.FLOOR.PRECISE(-5.5)</f>
@@ -2564,10 +2712,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="C4" s="4">
         <f>_xlfn.FLOOR.PRECISE(5.5,2)</f>
@@ -2579,10 +2727,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>238</v>
+        <v>267</v>
       </c>
       <c r="C5" s="4">
         <f>_xlfn.FLOOR.PRECISE(-5.5,2)</f>
@@ -2597,7 +2745,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
       <c r="C6" s="4">
         <f>_xlfn.FLOOR.PRECISE(0)</f>
@@ -2612,7 +2760,7 @@
         <v>57</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="C7" s="4">
         <f>_xlfn.FLOOR.PRECISE(3)</f>
@@ -2624,10 +2772,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="C8" s="4">
         <f>_xlfn.FLOOR.PRECISE(-0.1)</f>
@@ -2639,10 +2787,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="C9" s="4">
         <f>_xlfn.FLOOR.PRECISE(10,3)</f>
@@ -2657,7 +2805,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>_xlfn.FLOOR.PRECISE()</f>
@@ -2669,10 +2817,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="C11" s="10">
         <f>_xlfn.FLOOR.PRECISE(SQRT(10))</f>
@@ -2716,10 +2864,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="C2" s="4">
         <f>GCD(12,8)</f>
@@ -2731,10 +2879,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>250</v>
+        <v>279</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>251</v>
+        <v>280</v>
       </c>
       <c r="C3" s="4">
         <f>GCD(15,25)</f>
@@ -2746,10 +2894,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>252</v>
+        <v>281</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>253</v>
+        <v>282</v>
       </c>
       <c r="C4" s="4">
         <f>GCD(7,13)</f>
@@ -2761,10 +2909,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>255</v>
+        <v>284</v>
       </c>
       <c r="C5" s="4">
         <f>GCD(0,5)</f>
@@ -2776,10 +2924,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>256</v>
+        <v>285</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>257</v>
+        <v>286</v>
       </c>
       <c r="C6" s="4">
         <f>GCD(100,75,50)</f>
@@ -2791,10 +2939,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>258</v>
+        <v>287</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>259</v>
+        <v>288</v>
       </c>
       <c r="C7" s="4">
         <f>GCD(12,12)</f>
@@ -2806,10 +2954,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>260</v>
+        <v>289</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>261</v>
+        <v>290</v>
       </c>
       <c r="C8" s="4">
         <f>GCD(1,1)</f>
@@ -2821,10 +2969,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>262</v>
+        <v>291</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>263</v>
+        <v>292</v>
       </c>
       <c r="C9" s="4">
         <f>GCD(0,0)</f>
@@ -2839,7 +2987,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>GCD(-1,5)</f>
@@ -2854,7 +3002,7 @@
         <v>27</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
       <c r="C11" s="7" t="str">
         <f>GCD()</f>
@@ -2866,10 +3014,10 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>266</v>
+        <v>295</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
       <c r="C12" s="10">
         <f>GCD(LCM(4,6),12)</f>
@@ -2916,7 +3064,7 @@
         <v>49</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>268</v>
+        <v>297</v>
       </c>
       <c r="C2" s="4">
         <f>_xlfn.ISO.CEILING(5.5)</f>
@@ -2931,7 +3079,7 @@
         <v>51</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>269</v>
+        <v>298</v>
       </c>
       <c r="C3" s="4">
         <f>_xlfn.ISO.CEILING(-5.5)</f>
@@ -2946,7 +3094,7 @@
         <v>31</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="C4" s="4">
         <f>_xlfn.ISO.CEILING(5.5,2)</f>
@@ -2961,7 +3109,7 @@
         <v>54</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="C5" s="4">
         <f>_xlfn.ISO.CEILING(-5.5,2)</f>
@@ -2976,7 +3124,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="C6" s="4">
         <f>_xlfn.ISO.CEILING(0)</f>
@@ -2991,7 +3139,7 @@
         <v>57</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="C7" s="4">
         <f>_xlfn.ISO.CEILING(3)</f>
@@ -3006,7 +3154,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>274</v>
+        <v>303</v>
       </c>
       <c r="C8" s="4">
         <f>_xlfn.ISO.CEILING(-0.1,1)</f>
@@ -3021,7 +3169,7 @@
         <v>59</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="C9" s="4">
         <f>_xlfn.ISO.CEILING(-3)</f>
@@ -3036,7 +3184,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>_xlfn.ISO.CEILING()</f>
@@ -3048,10 +3196,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>277</v>
+        <v>306</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>278</v>
+        <v>307</v>
       </c>
       <c r="C11" s="10">
         <f>_xlfn.ISO.CEILING(PI())</f>
@@ -3095,10 +3243,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>308</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>280</v>
+        <v>309</v>
       </c>
       <c r="C2" s="4">
         <f>LCM(4,6)</f>
@@ -3110,10 +3258,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>281</v>
+        <v>310</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>282</v>
+        <v>311</v>
       </c>
       <c r="C3" s="4">
         <f>LCM(5,3)</f>
@@ -3125,10 +3273,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>283</v>
+        <v>312</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>284</v>
+        <v>313</v>
       </c>
       <c r="C4" s="4">
         <f>LCM(7,7)</f>
@@ -3140,10 +3288,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>285</v>
+        <v>314</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>286</v>
+        <v>315</v>
       </c>
       <c r="C5" s="4">
         <f>LCM(1,5)</f>
@@ -3155,10 +3303,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>287</v>
+        <v>316</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>288</v>
+        <v>317</v>
       </c>
       <c r="C6" s="4">
         <f>LCM(12,8,6)</f>
@@ -3170,10 +3318,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>289</v>
+        <v>318</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>290</v>
+        <v>319</v>
       </c>
       <c r="C7" s="4">
         <f>LCM(1,1)</f>
@@ -3185,10 +3333,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>291</v>
+        <v>320</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>292</v>
+        <v>321</v>
       </c>
       <c r="C8" s="4">
         <f>LCM(7,1)</f>
@@ -3200,10 +3348,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>293</v>
+        <v>322</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>294</v>
+        <v>323</v>
       </c>
       <c r="C9" s="4">
         <f>LCM(0,5)</f>
@@ -3218,7 +3366,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>295</v>
+        <v>324</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>LCM(-1,5)</f>
@@ -3233,7 +3381,7 @@
         <v>27</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>296</v>
+        <v>325</v>
       </c>
       <c r="C11" s="7" t="str">
         <f>LCM()</f>
@@ -3245,10 +3393,10 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>297</v>
+        <v>326</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>298</v>
+        <v>327</v>
       </c>
       <c r="C12" s="10">
         <f>LCM(GCD(12,8),6)</f>
@@ -3292,10 +3440,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>299</v>
+        <v>328</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>300</v>
+        <v>329</v>
       </c>
       <c r="C2" s="4">
         <f>MULTINOMIAL(2,3)</f>
@@ -3307,10 +3455,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>301</v>
+        <v>330</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>302</v>
+        <v>331</v>
       </c>
       <c r="C3" s="4">
         <f>MULTINOMIAL(1,1,1)</f>
@@ -3322,10 +3470,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>303</v>
+        <v>332</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>304</v>
+        <v>333</v>
       </c>
       <c r="C4" s="4">
         <f>MULTINOMIAL(4)</f>
@@ -3337,10 +3485,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>305</v>
+        <v>334</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>306</v>
+        <v>335</v>
       </c>
       <c r="C5" s="4">
         <f>MULTINOMIAL(3,2,1)</f>
@@ -3352,10 +3500,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>307</v>
+        <v>336</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>308</v>
+        <v>337</v>
       </c>
       <c r="C6" s="4">
         <f>MULTINOMIAL(1,2)</f>
@@ -3367,10 +3515,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>309</v>
+        <v>338</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>310</v>
+        <v>339</v>
       </c>
       <c r="C7" s="4">
         <f>MULTINOMIAL(0,3)</f>
@@ -3382,10 +3530,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>311</v>
+        <v>340</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>312</v>
+        <v>341</v>
       </c>
       <c r="C8" s="4">
         <f>MULTINOMIAL(2,2,2)</f>
@@ -3400,7 +3548,7 @@
         <v>25</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>313</v>
+        <v>342</v>
       </c>
       <c r="C9" s="7" t="str">
         <f>MULTINOMIAL(-1,2)</f>
@@ -3415,7 +3563,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>314</v>
+        <v>343</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>MULTINOMIAL()</f>
@@ -3427,10 +3575,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>315</v>
+        <v>344</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>316</v>
+        <v>345</v>
       </c>
       <c r="C11" s="10" t="b">
         <f>IF(MULTINOMIAL(2,3)=COMBIN(5,2),TRUE,FALSE)</f>
@@ -3474,10 +3622,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>317</v>
+        <v>346</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>318</v>
+        <v>347</v>
       </c>
       <c r="C2" s="4" t="b">
         <f>ISNUMBER(RAND())</f>
@@ -3489,10 +3637,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>319</v>
+        <v>348</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>320</v>
+        <v>349</v>
       </c>
       <c r="C3" s="4" t="b">
         <f>RAND()&gt;=0</f>
@@ -3504,10 +3652,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>321</v>
+        <v>350</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>322</v>
+        <v>351</v>
       </c>
       <c r="C4" s="4" t="b">
         <f>RAND()&lt;1</f>
@@ -3519,10 +3667,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>323</v>
+        <v>352</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="C5" s="4" t="b">
         <f>INT(RAND()*100)&gt;=0</f>
@@ -3534,10 +3682,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>325</v>
+        <v>354</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>326</v>
+        <v>355</v>
       </c>
       <c r="C6" s="4" t="b">
         <f>INT(RAND()*100)&lt;100</f>
@@ -3549,10 +3697,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>327</v>
+        <v>356</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>328</v>
+        <v>357</v>
       </c>
       <c r="C7" s="4">
         <f>RAND()*0</f>
@@ -3564,10 +3712,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>329</v>
+        <v>358</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>330</v>
+        <v>359</v>
       </c>
       <c r="C8" s="4" t="b">
         <f>ISNUMBER(RAND()+0)</f>
@@ -3579,10 +3727,10 @@
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>331</v>
+        <v>360</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>332</v>
+        <v>361</v>
       </c>
       <c r="C9" s="10" t="b">
         <f>AND(RAND()&gt;=0,RAND()&lt;1)</f>
@@ -3626,10 +3774,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>333</v>
+        <v>362</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>334</v>
+        <v>363</v>
       </c>
       <c r="C2" s="4" t="b">
         <f>ISNUMBER(RANDBETWEEN(1,10))</f>
@@ -3641,10 +3789,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>335</v>
+        <v>364</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>336</v>
+        <v>365</v>
       </c>
       <c r="C3" s="4">
         <f>RANDBETWEEN(5,5)</f>
@@ -3656,10 +3804,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>337</v>
+        <v>366</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>338</v>
+        <v>367</v>
       </c>
       <c r="C4" s="4">
         <f>RANDBETWEEN(0,0)</f>
@@ -3671,10 +3819,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>339</v>
+        <v>368</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>340</v>
+        <v>369</v>
       </c>
       <c r="C5" s="4" t="b">
         <f>RANDBETWEEN(1,100)&gt;=1</f>
@@ -3686,10 +3834,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>341</v>
+        <v>370</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>342</v>
+        <v>371</v>
       </c>
       <c r="C6" s="4" t="b">
         <f>RANDBETWEEN(1,100)&lt;=100</f>
@@ -3701,10 +3849,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>343</v>
+        <v>372</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>344</v>
+        <v>373</v>
       </c>
       <c r="C7" s="4" t="b">
         <f>RANDBETWEEN(-10,10)&lt;=10</f>
@@ -3716,10 +3864,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>345</v>
+        <v>374</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>346</v>
+        <v>375</v>
       </c>
       <c r="C8" s="4">
         <f>RANDBETWEEN(-5,-5)</f>
@@ -3731,10 +3879,10 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>347</v>
+        <v>376</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>348</v>
+        <v>377</v>
       </c>
       <c r="C9" s="7" t="str">
         <f>RANDBETWEEN(5,3)</f>
@@ -3749,7 +3897,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>349</v>
+        <v>378</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>RANDBETWEEN()</f>
@@ -3761,10 +3909,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>350</v>
+        <v>379</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>351</v>
+        <v>380</v>
       </c>
       <c r="C11" s="10" t="b">
         <f>AND(RANDBETWEEN(1,100)&gt;=1,RANDBETWEEN(1,100)&lt;=100)</f>
@@ -3990,10 +4138,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>352</v>
+        <v>381</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>353</v>
+        <v>382</v>
       </c>
       <c r="C2" s="4">
         <f t="array" ref="C2">SERIESSUM(1,0,1,1)</f>
@@ -4005,10 +4153,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>354</v>
+        <v>383</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>355</v>
+        <v>384</v>
       </c>
       <c r="C3" s="4">
         <f t="array" ref="C3">SERIESSUM(2,1,1,{1,1})</f>
@@ -4020,10 +4168,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>356</v>
+        <v>385</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>357</v>
+        <v>386</v>
       </c>
       <c r="C4" s="4">
         <f t="array" ref="C4">SERIESSUM(1,0,1,{1,1})</f>
@@ -4035,10 +4183,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>358</v>
+        <v>387</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>359</v>
+        <v>388</v>
       </c>
       <c r="C5" s="4">
         <f t="array" ref="C5">SERIESSUM(3,0,0,5)</f>
@@ -4050,10 +4198,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>360</v>
+        <v>389</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>361</v>
+        <v>390</v>
       </c>
       <c r="C6" s="4">
         <f t="array" ref="C6">SERIESSUM(0,1,1,{5,3})</f>
@@ -4065,10 +4213,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>362</v>
+        <v>391</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>363</v>
+        <v>392</v>
       </c>
       <c r="C7" s="4">
         <f t="array" ref="C7">SERIESSUM(1,1,1,{1,1,1})</f>
@@ -4080,10 +4228,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>365</v>
+        <v>394</v>
       </c>
       <c r="C8" s="4">
         <f t="array" ref="C8">SERIESSUM(2,0,2,{1,1})</f>
@@ -4095,10 +4243,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>366</v>
+        <v>395</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>367</v>
+        <v>396</v>
       </c>
       <c r="C9" s="4">
         <f t="array" ref="C9">SERIESSUM(10,0,1,1)</f>
@@ -4113,7 +4261,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>368</v>
+        <v>397</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>SERIESSUM()</f>
@@ -4125,10 +4273,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>369</v>
+        <v>398</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>370</v>
+        <v>399</v>
       </c>
       <c r="C11" s="10">
         <f t="array" ref="C11">ROUND(SERIESSUM(1,0,1,{1,1,0.5}),2)</f>
@@ -4172,10 +4320,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>371</v>
+        <v>400</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>372</v>
+        <v>401</v>
       </c>
       <c r="C2" s="4">
         <f>ROUND(SQRTPI(1),6)</f>
@@ -4187,10 +4335,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>373</v>
+        <v>402</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>374</v>
+        <v>403</v>
       </c>
       <c r="C3" s="4">
         <f>ROUND(SQRTPI(4),6)</f>
@@ -4202,10 +4350,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>375</v>
+        <v>404</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>376</v>
+        <v>405</v>
       </c>
       <c r="C4" s="4">
         <f>SQRTPI(0)</f>
@@ -4217,10 +4365,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>377</v>
+        <v>406</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>378</v>
+        <v>407</v>
       </c>
       <c r="C5" s="4">
         <f>ROUND(SQRTPI(1/PI()),10)</f>
@@ -4232,10 +4380,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>379</v>
+        <v>408</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>380</v>
+        <v>409</v>
       </c>
       <c r="C6" s="4">
         <f>ROUND(SQRTPI(PI()),6)</f>
@@ -4247,10 +4395,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>381</v>
+        <v>410</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>382</v>
+        <v>411</v>
       </c>
       <c r="C7" s="4">
         <f>ROUND(SQRTPI(9),5)</f>
@@ -4262,10 +4410,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>383</v>
+        <v>412</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>384</v>
+        <v>413</v>
       </c>
       <c r="C8" s="4">
         <f>ROUND(SQRTPI(0.25),6)</f>
@@ -4280,7 +4428,7 @@
         <v>25</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>385</v>
+        <v>414</v>
       </c>
       <c r="C9" s="7" t="str">
         <f>SQRTPI(-1)</f>
@@ -4295,7 +4443,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>386</v>
+        <v>415</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>SQRTPI()</f>
@@ -4307,10 +4455,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>387</v>
+        <v>416</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>388</v>
+        <v>417</v>
       </c>
       <c r="C11" s="10">
         <f>ROUND(SQRTPI(1)^2,6)</f>
@@ -4332,10 +4480,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="27.13"/>
-    <col customWidth="1" min="2" max="2" width="37.25"/>
+    <col customWidth="1" min="1" max="1" width="30.25"/>
+    <col customWidth="1" min="2" max="2" width="39.13"/>
     <col customWidth="1" min="3" max="3" width="14.13"/>
-    <col customWidth="1" min="4" max="4" width="5.88"/>
+    <col customWidth="1" min="4" max="4" width="7.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4354,10 +4502,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>389</v>
+        <v>418</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>390</v>
+        <v>419</v>
       </c>
       <c r="C2" s="4">
         <f t="array" ref="C2">SUMIF({1,2,3,4,5},"&gt;"&amp;2)</f>
@@ -4369,10 +4517,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>391</v>
+        <v>420</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>392</v>
+        <v>421</v>
       </c>
       <c r="C3" s="4" t="str">
         <f t="array" ref="C3">SUMIF({1,2,3},"&gt;="&amp;2,{10,20,30})</f>
@@ -4384,10 +4532,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>393</v>
+        <v>422</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>394</v>
+        <v>423</v>
       </c>
       <c r="C4" s="4" t="str">
         <f t="array" ref="C4">SUMIF({"a","b","a"},"a",{1,2,3})</f>
@@ -4399,10 +4547,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>395</v>
+        <v>424</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>396</v>
+        <v>425</v>
       </c>
       <c r="C5" s="4">
         <f t="array" ref="C5">SUMIF({1,2,3,4,5},"&lt;="&amp;2)</f>
@@ -4414,10 +4562,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>397</v>
+        <v>426</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>398</v>
+        <v>427</v>
       </c>
       <c r="C6" s="4">
         <f t="array" ref="C6">SUMIF({1,2,3,4,5},3)</f>
@@ -4429,76 +4577,151 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>135</v>
+        <v>428</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="C7" s="4">
-        <f t="array" ref="C7">SUMIF({1,2,3},"&gt;"&amp;10)</f>
-        <v>0</v>
+        <f t="array" ref="C7">SUMIF({1,2,3},"&lt;&gt;"&amp;2)</f>
+        <v>4</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="C8" s="4" t="str">
-        <f t="array" ref="C8">SUMIF({"a","b","c"},"*",{10,20,30})</f>
-        <v>#N/A</v>
+        <v>430</v>
+      </c>
+      <c r="C8" s="4">
+        <f t="array" ref="C8">SUMIF({1,2,3},"&gt;"&amp;10)</f>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="C9" s="4" t="str">
+        <f t="array" ref="C9">SUMIF({"a","b","c"},"*",{10,20,30})</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="C10" s="4" t="str">
+        <f t="array" ref="C10">SUMIF({"ab","ac","ba"},"a?",{10,20,30})</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="C11" s="4" t="str">
+        <f t="array" ref="C11">SUMIF({"Apple","APPLE","banana"},"apple",{10,20,30})</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>438</v>
+      </c>
+      <c r="C12" s="13" t="str">
+        <f t="array" ref="C12">SUMIF({1,2,3},"2",{10,20,30})</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>402</v>
-      </c>
-      <c r="C9" s="7" t="str">
+      <c r="B13" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="C13" s="7" t="str">
         <f>SUMIF()</f>
         <v>#N/A</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>404</v>
-      </c>
-      <c r="C10" s="10">
-        <f t="array" ref="C10">SUMIF({1,2,3,4,5},"&gt;"&amp;3)+SUMIF({1,2,3,4,5},"&lt;="&amp;2)</f>
+    <row r="14">
+      <c r="A14" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="C14" s="10">
+        <f t="array" ref="C14">SUMIF({1,2,3,4,5},"&gt;"&amp;3)+SUMIF({1,2,3,4,5},"&lt;="&amp;2)</f>
         <v>12</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D14" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>405</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>406</v>
-      </c>
-      <c r="C11" s="10" t="str">
-        <f t="array" ref="C11">SUMIF({1,2,3},"&gt;"&amp;1,{-10,-20,-30})</f>
+    <row r="15">
+      <c r="A15" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="C15" s="10" t="str">
+        <f t="array" ref="C15">SUMIF({1,2,3},"&gt;"&amp;1,{-10,-20,-30})</f>
         <v>#N/A</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D15" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="C16" s="10" t="str">
+        <f t="array" ref="C16">ROUND(SUMIF({1.1,2.2,3.3},"&gt;"&amp;2,{10,20,30}),0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>48</v>
       </c>
     </row>
@@ -4514,7 +4737,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.75"/>
+    <col customWidth="1" min="1" max="1" width="24.0"/>
     <col customWidth="1" min="2" max="2" width="52.88"/>
     <col customWidth="1" min="3" max="3" width="14.13"/>
     <col customWidth="1" min="4" max="4" width="5.88"/>
@@ -4536,10 +4759,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>407</v>
+        <v>446</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>408</v>
+        <v>447</v>
       </c>
       <c r="C2" s="4" t="str">
         <f t="array" ref="C2">SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;2)</f>
@@ -4551,10 +4774,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>409</v>
+        <v>448</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>410</v>
+        <v>449</v>
       </c>
       <c r="C3" s="4" t="str">
         <f t="array" ref="C3">SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;1,{1,2,3,4,5},"&lt;"&amp;5)</f>
@@ -4566,10 +4789,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>393</v>
+        <v>422</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>411</v>
+        <v>450</v>
       </c>
       <c r="C4" s="4" t="str">
         <f t="array" ref="C4">SUMIFS({10,20,30},{"a","b","a"},"a")</f>
@@ -4581,10 +4804,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>412</v>
+        <v>451</v>
       </c>
       <c r="C5" s="4" t="str">
         <f t="array" ref="C5">SUMIFS({1,2,3},{1,2,3},"&gt;"&amp;10)</f>
@@ -4596,61 +4819,106 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>413</v>
+        <v>452</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>414</v>
+        <v>453</v>
       </c>
       <c r="C6" s="4" t="str">
-        <f t="array" ref="C6">SUMIFS({10,20,30},{1,2,3},2)</f>
+        <f t="array" ref="C6">SUMIFS({10,20,30},{1,2,3},"&lt;&gt;"&amp;2)</f>
         <v>#N/A</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="C7" s="4" t="str">
+        <f t="array" ref="C7">SUMIFS({10,20,30},{1,2,3},2)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="s">
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="C8" s="4" t="str">
+        <f t="array" ref="C8">SUMIFS({10,20,30},{"apple","apricot","banana"},"a*")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="C9" s="4" t="str">
+        <f t="array" ref="C9">SUMIFS({100,200,300,400},{"a","b","a","b"},"a",{1,2,1,2},1)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>415</v>
-      </c>
-      <c r="C7" s="7" t="str">
+      <c r="B10" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="C10" s="7" t="str">
         <f>SUMIFS()</f>
         <v>#N/A</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="s">
-        <v>416</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="C8" s="10" t="str">
-        <f t="array" ref="C8">SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;3)+SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&lt;"&amp;3)</f>
+    <row r="11">
+      <c r="A11" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="C11" s="10" t="str">
+        <f t="array" ref="C11">SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;3)+SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&lt;"&amp;3)</f>
         <v>#N/A</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="s">
-        <v>418</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="C9" s="10" t="str">
-        <f t="array" ref="C9">SUMIFS({100,200,300,400},{"a","b","a","b"},"a",{1,2,1,2},1)</f>
+    <row r="12">
+      <c r="A12" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="C12" s="10" t="str">
+        <f t="array" ref="C12">ROUND(SUMIFS({1,2,3,4,5},{1,2,3,4,5},"&gt;"&amp;1,{1,2,3,4,5},"&lt;"&amp;5),0)</f>
         <v>#N/A</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D12" s="8" t="s">
         <v>48</v>
       </c>
     </row>
@@ -4688,10 +4956,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>420</v>
+        <v>465</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>421</v>
+        <v>466</v>
       </c>
       <c r="C2" s="4">
         <f>SUMSQ(3,4)</f>
@@ -4703,10 +4971,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>422</v>
+        <v>467</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="C3" s="4">
         <f>SUMSQ(1,2,3)</f>
@@ -4718,10 +4986,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>424</v>
+        <v>469</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>425</v>
+        <v>470</v>
       </c>
       <c r="C4" s="4">
         <f t="array" ref="C4">SUMSQ({1,2,3,4})</f>
@@ -4733,10 +5001,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>426</v>
+        <v>471</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>427</v>
+        <v>472</v>
       </c>
       <c r="C5" s="4">
         <f>SUMSQ(5)</f>
@@ -4748,10 +5016,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>428</v>
+        <v>473</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>429</v>
+        <v>474</v>
       </c>
       <c r="C6" s="4">
         <f>SUMSQ(0)</f>
@@ -4763,10 +5031,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>430</v>
+        <v>475</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>431</v>
+        <v>476</v>
       </c>
       <c r="C7" s="4">
         <f>SUMSQ(1,1,1,1,1)</f>
@@ -4778,10 +5046,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>432</v>
+        <v>477</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>433</v>
+        <v>478</v>
       </c>
       <c r="C8" s="4">
         <f>SUMSQ(-3,-4)</f>
@@ -4793,10 +5061,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>434</v>
+        <v>479</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>435</v>
+        <v>480</v>
       </c>
       <c r="C9" s="4">
         <f>SUMSQ(0.5,0.5)</f>
@@ -4811,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>436</v>
+        <v>481</v>
       </c>
       <c r="C10" s="7" t="str">
         <f>SUMSQ()</f>
@@ -4823,10 +5091,10 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>437</v>
+        <v>482</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>438</v>
+        <v>483</v>
       </c>
       <c r="C11" s="10">
         <f>SQRT(SUMSQ(3,4))</f>
@@ -4838,10 +5106,10 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>439</v>
+        <v>484</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>440</v>
+        <v>485</v>
       </c>
       <c r="C12" s="10">
         <f>SUMSQ(SQRT(2),SQRT(2))</f>
@@ -5425,9 +5693,9 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="32.38"/>
-    <col customWidth="1" min="2" max="2" width="29.75"/>
+    <col customWidth="1" min="2" max="2" width="33.13"/>
     <col customWidth="1" min="3" max="3" width="14.13"/>
-    <col customWidth="1" min="4" max="4" width="5.88"/>
+    <col customWidth="1" min="4" max="4" width="7.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5550,32 +5818,122 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" s="4">
+        <f t="array" ref="C9">COUNTBLANK(0)</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" s="4">
+        <f t="array" ref="C10">COUNTBLANK(FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="4">
+        <f t="array" ref="C11">COUNTBLANK(TRUE)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="array" ref="C12">COUNTBLANK({"hello","","world"})</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="13">
+        <f t="array" ref="C13">COUNTBLANK({TRUE,FALSE,""})</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C9" s="7" t="str">
+      <c r="B14" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C14" s="7" t="str">
         <f>COUNTBLANK()</f>
         <v>#N/A</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="C10" s="10">
-        <f t="array" ref="C10">COUNTBLANK({"",1,"",2})+COUNT({1,2})</f>
+    <row r="15">
+      <c r="A15" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="C15" s="10">
+        <f t="array" ref="C15">COUNTBLANK({"",1,"",2})+COUNT({1,2})</f>
         <v>4</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D15" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C16" s="10">
+        <f t="array" ref="C16">COUNTBLANK({"",1,"",2})+COUNTA({"",1,"",2})</f>
+        <v>6</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>48</v>
       </c>
     </row>
@@ -5591,10 +5949,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="28.0"/>
-    <col customWidth="1" min="2" max="2" width="29.38"/>
+    <col customWidth="1" min="1" max="1" width="37.0"/>
+    <col customWidth="1" min="2" max="2" width="41.13"/>
     <col customWidth="1" min="3" max="3" width="14.13"/>
-    <col customWidth="1" min="4" max="4" width="5.88"/>
+    <col customWidth="1" min="4" max="4" width="7.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5613,10 +5971,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="C2" s="4">
         <f t="array" ref="C2">COUNTIF({1,2,3,4,5},"&gt;"&amp;2)</f>
@@ -5628,10 +5986,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="C3" s="4">
         <f t="array" ref="C3">COUNTIF({1,2,3,2,1},2)</f>
@@ -5643,10 +6001,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="C4" s="4">
         <f t="array" ref="C4">COUNTIF({"a","b","a","c"},"a")</f>
@@ -5658,10 +6016,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="C5" s="4">
         <f t="array" ref="C5">COUNTIF({1,2,3,4,5},"&lt;="&amp;3)</f>
@@ -5673,10 +6031,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="C6" s="4">
         <f t="array" ref="C6">COUNTIF({1,2,3,4,5},"&gt;="&amp;2)</f>
@@ -5688,14 +6046,14 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C7" s="4">
-        <f t="array" ref="C7">COUNTIF({1,2,3,4,5},"*")</f>
-        <v>0</v>
+        <f t="array" ref="C7">COUNTIF({"a","b","c"},"*")</f>
+        <v>3</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>6</v>
@@ -5703,61 +6061,136 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="C8" s="4">
-        <f t="array" ref="C8">COUNTIF({1,2,3},"&gt;10")</f>
-        <v>0</v>
+        <f t="array" ref="C8">COUNTIF({1,2,3,2,1},"&lt;&gt;"&amp;2)</f>
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="C9" s="4">
-        <f t="array" ref="C9">COUNTIF({TRUE,FALSE,FALSE},FALSE)</f>
-        <v>2</v>
+        <f t="array" ref="C9">COUNTIF({1,2,3},"&gt;10")</f>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="4">
+        <f t="array" ref="C10">COUNTIF({TRUE,FALSE,FALSE},FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11" s="4">
+        <f t="array" ref="C11">COUNTIF({"apt","ape","app","bat"},"ap?")</f>
+        <v>3</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="array" ref="C12">COUNTIF({"a","b","A","c"},"a")</f>
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" s="13">
+        <f t="array" ref="C13">COUNTIF({1,2,3},2)</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C10" s="7" t="str">
+      <c r="B14" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C14" s="7" t="str">
         <f>COUNTIF()</f>
         <v>#N/A</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="C11" s="10">
-        <f t="array" ref="C11">COUNTIF({1,2,3,4,5},"&gt;"&amp;2)*2</f>
-        <v>6</v>
-      </c>
-      <c r="D11" s="8" t="s">
+    <row r="15">
+      <c r="A15" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C15" s="10">
+        <f t="array" ref="C15">COUNTIF({1,2,3,4,5},"&gt;"&amp;2)*2</f>
+        <v>6</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C16" s="10">
+        <f t="array" ref="C16">COUNTIF({1,2,3,4,5},"&gt;"&amp;2)+COUNTIF({1,2,3,4,5},"&lt;="&amp;2)</f>
+        <v>5</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>48</v>
       </c>
     </row>
@@ -5773,7 +6206,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="22.88"/>
+    <col customWidth="1" min="1" max="1" width="25.88"/>
     <col customWidth="1" min="2" max="2" width="42.13"/>
     <col customWidth="1" min="3" max="3" width="14.13"/>
     <col customWidth="1" min="4" max="4" width="5.88"/>
@@ -5795,10 +6228,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="C2" s="4">
         <f t="array" ref="C2">COUNTIFS({1,2,3,4,5},"&gt;"&amp;2)</f>
@@ -5810,10 +6243,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="C3" s="4">
         <f t="array" ref="C3">COUNTIFS({1,2,3,4,5},"&gt;"&amp;1,{1,2,3,4,5},"&lt;"&amp;5)</f>
@@ -5825,10 +6258,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="C4" s="4">
         <f t="array" ref="C4">COUNTIFS({1,2,3},"&gt;"&amp;5,{1,2,3},"&lt;"&amp;10)</f>
@@ -5840,10 +6273,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>148</v>
+        <v>171</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>149</v>
+        <v>172</v>
       </c>
       <c r="C5" s="4">
         <f t="array" ref="C5">COUNTIFS({1,2,3,2,1},2)</f>
@@ -5855,62 +6288,107 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
       <c r="C6" s="4">
-        <f t="array" ref="C6">COUNTIFS({1,2,3},"&gt;="&amp;1,{1,2,3},"&lt;="&amp;3)</f>
+        <f t="array" ref="C6">COUNTIFS({1,2,3,2,1},"&lt;&gt;"&amp;2)</f>
         <v>3</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" s="4">
+        <f t="array" ref="C7">COUNTIFS({1,2,3},"&gt;="&amp;1,{1,2,3},"&lt;="&amp;3)</f>
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="s">
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C8" s="4">
+        <f t="array" ref="C8">COUNTIFS({"a","b","a","c"},"a")</f>
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C9" s="4">
+        <f t="array" ref="C9">COUNTIFS({"apple","apricot","banana"},"a*")</f>
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C7" s="7" t="str">
+      <c r="B10" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C10" s="7" t="str">
         <f>COUNTIFS()</f>
         <v>#N/A</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="C8" s="10">
-        <f t="array" ref="C8">COUNTIFS({1,2,3,4,5},"&gt;"&amp;2)+COUNTIFS({1,2,3,4,5},"&lt;"&amp;3)</f>
+    <row r="11">
+      <c r="A11" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="C11" s="10">
+        <f t="array" ref="C11">COUNTIFS({1,2,3,4,5},"&gt;"&amp;2)+COUNTIFS({1,2,3,4,5},"&lt;"&amp;3)</f>
         <v>5</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C9" s="4">
-        <f t="array" ref="C9">COUNTIFS({"a","b","a","c"},"a")</f>
-        <v>2</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>6</v>
+    <row r="12">
+      <c r="A12" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="C12" s="10" t="str">
+        <f t="array" ref="C12">IF(COUNTIFS({1,2,3,4,5},"&gt;"&amp;4)=1,"yes","no")</f>
+        <v>yes</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -5947,10 +6425,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="C2" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE(1,2,2,3,3,3)"),3.0)</f>
@@ -5962,10 +6440,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="C3" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE(""a"",""b"",""a"")"),2.0)</f>
@@ -5977,10 +6455,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="C4" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE(1)"),1.0)</f>
@@ -5992,10 +6470,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
       <c r="C5" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE({1,2,2,3})"),3.0)</f>
@@ -6007,10 +6485,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>165</v>
+        <v>194</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>166</v>
+        <v>195</v>
       </c>
       <c r="C6" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE(5,5,5)"),1.0)</f>
@@ -6022,10 +6500,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>167</v>
+        <v>196</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="C7" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE(1,2,3,4,5)"),5.0)</f>
@@ -6037,10 +6515,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="C8" s="4">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE(1,""1"",TRUE)"),3.0)</f>
@@ -6055,7 +6533,7 @@
         <v>27</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C9" s="7" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("COUNTUNIQUE()"),"#N/A")</f>
@@ -6067,10 +6545,10 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>172</v>
+        <v>201</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="C10" s="10" t="b">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IF(COUNTUNIQUE(1,2,2,3)=3,TRUE,FALSE)"),TRUE)</f>

</xml_diff>